<commit_message>
docs: update author to Lai Thi Thanh Xuan (23110309), deploy link onrender.com, and Google Drive links
</commit_message>
<xml_diff>
--- a/docs/Mau_02_Bug_Manifest.xlsx
+++ b/docs/Mau_02_Bug_Manifest.xlsx
@@ -542,7 +542,7 @@
       <c r="B4" s="14" t="n"/>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Sinh viên A</t>
+          <t>Lại Thị Thanh Xuân</t>
         </is>
       </c>
       <c r="D4" s="15" t="n"/>
@@ -577,7 +577,7 @@
       <c r="B5" s="14" t="n"/>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>SV20260001</t>
+          <t>23110309</t>
         </is>
       </c>
       <c r="D5" s="15" t="n"/>
@@ -639,7 +639,7 @@
       <c r="B7" s="14" t="n"/>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>http://127.0.0.1:8001</t>
+          <t>https://itick-platform.onrender.com/ (Local: http://127.0.0.1:8001)</t>
         </is>
       </c>
       <c r="D7" s="15" t="n"/>
@@ -701,7 +701,7 @@
       <c r="B9" s="14" t="n"/>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Tuần 6</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="D9" s="15" t="n"/>
@@ -724,6 +724,16 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Link Drive minh chứng Bug (Bí mật)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1K9Mq0RubxVY5YOycdWN-DqwUO4dmS-kc?usp=sharing</t>
+        </is>
+      </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Tổng số lỗi</t>
@@ -742,6 +752,16 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mã nguồn GitHub</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://github.com/DYouth572/itick-platform</t>
+        </is>
+      </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Mức Critical + Major</t>
@@ -2263,14 +2283,14 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A9:B9"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A8:B8"/>
     <mergeCell ref="C7:E7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:E6"/>
   </mergeCells>
   <conditionalFormatting sqref="J5:J11">

</xml_diff>